<commit_message>
Update LED9101 firmware docs and timing
</commit_message>
<xml_diff>
--- a/CIU32F003F5P6-TSSOP20.xlsx
+++ b/CIU32F003F5P6-TSSOP20.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet name="CIU32F003F5P6-TSSOP20" sheetId="1" r:id="rId1"/>
     <sheet name="CIU32F003F5P6-SOP8" sheetId="4" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="端口复用" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="92">
   <si>
     <t>PIN</t>
   </si>
@@ -77,6 +77,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve">SPI1_NSS
 </t>
     </r>
@@ -142,6 +149,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve">SPI1_MOSI
 </t>
     </r>
@@ -220,6 +234,9 @@
     <t>采样pwm信号的频率和占空比，频率允许800Hz-24K</t>
   </si>
   <si>
+    <t>真实的8P用</t>
+  </si>
+  <si>
     <t>PC0</t>
   </si>
   <si>
@@ -237,6 +254,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve">SPI1_MISO
 </t>
     </r>
@@ -253,10 +277,26 @@
     </r>
   </si>
   <si>
+    <t>Tim1_CH2</t>
+  </si>
+  <si>
+    <t>测试用，直接连在in2</t>
+  </si>
+  <si>
+    <t>PC1-&gt;PA7</t>
+  </si>
+  <si>
     <t>PB7</t>
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve">SPI1_MOSI
 </t>
     </r>
@@ -293,6 +333,15 @@
       </rPr>
       <t>TIM1_CH4</t>
     </r>
+  </si>
+  <si>
+    <t>Tim1_ch4</t>
+  </si>
+  <si>
+    <t>测试用，跟随PWM_IN2,输出对应的占空比，频率16K</t>
+  </si>
+  <si>
+    <t>调试用，8P的脚刚好有电容</t>
   </si>
   <si>
     <t>VSS</t>
@@ -328,6 +377,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve">SPI1_NSS
 </t>
     </r>
@@ -371,6 +426,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>UART1_TX</t>
     </r>
     <r>
@@ -425,6 +487,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve">SPI1_SCK
 </t>
     </r>
@@ -483,7 +552,7 @@
     </r>
   </si>
   <si>
-    <t>TIM1_CH1</t>
+    <t>TIM1_CH3</t>
   </si>
   <si>
     <t>PWM1</t>
@@ -501,6 +570,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve">SPI1_NSS
 TIM1_CH1N
 TIM1_CH2N
@@ -529,7 +605,7 @@
     </r>
   </si>
   <si>
-    <t>TIM1_CH2N</t>
+    <t>TIM1_CH4</t>
   </si>
   <si>
     <t>PWM2</t>
@@ -546,6 +622,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve">SPI1_SCK
 </t>
     </r>
@@ -593,6 +676,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve">SPI1_MOSI
 </t>
     </r>
@@ -621,10 +711,26 @@
     </r>
   </si>
   <si>
+    <t>TIm_ch1</t>
+  </si>
+  <si>
+    <t>测试用，直接连在in1</t>
+  </si>
+  <si>
+    <t>PA0--&gt;PB0</t>
+  </si>
+  <si>
     <t>PA1</t>
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve">SPI1_MISO
 </t>
     </r>
@@ -639,6 +745,12 @@
       <t>TIM1_CH2
 TIM1_CH3</t>
     </r>
+  </si>
+  <si>
+    <t>Tim1_ch3</t>
+  </si>
+  <si>
+    <t>测试用，跟随PWM_IN1,输出对应的占空比，频率16K</t>
   </si>
   <si>
     <t>PA2</t>
@@ -662,6 +774,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>UART1_TX</t>
     </r>
     <r>
@@ -722,6 +841,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>UART1_RX</t>
     </r>
     <r>
@@ -769,6 +895,12 @@
   <si>
     <t>UART1_RX
 /UART2_TX</t>
+  </si>
+  <si>
+    <t>TIM1_CH1</t>
+  </si>
+  <si>
+    <t>TIM1_CH2N</t>
   </si>
   <si>
     <t>SWCLK
@@ -785,7 +917,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="25">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -802,13 +934,20 @@
     </font>
     <font>
       <sz val="11"/>
+      <color rgb="FF0070C0"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color theme="0" tint="-0.15"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0" tint="-0.25"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -965,18 +1104,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="35">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -1310,137 +1443,137 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1475,9 +1608,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1485,30 +1615,39 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1574,6 +1713,95 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="图片 1"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2057400" y="342900"/>
+          <a:ext cx="9620250" cy="6877050"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>600075</xdr:colOff>
+      <xdr:row>58</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="图片 2"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2057400" y="7372350"/>
+          <a:ext cx="9515475" cy="2724150"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1918,7 +2146,7 @@
       <c r="E2" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="15"/>
+      <c r="F2" s="14"/>
       <c r="G2" s="4"/>
       <c r="H2" s="6"/>
       <c r="I2" s="6"/>
@@ -1939,8 +2167,8 @@
       <c r="E3" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="F3" s="15"/>
-      <c r="G3" s="15"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
       <c r="H3" s="9"/>
       <c r="I3" s="6"/>
     </row>
@@ -1960,35 +2188,37 @@
       <c r="E4" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="G4" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="H4" s="9" t="s">
+      <c r="H4" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="I4" s="6"/>
+      <c r="I4" s="16" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="5" ht="27" spans="1:9">
       <c r="A5" s="10">
         <v>4</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C5" s="10" t="s">
         <v>10</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="E5" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="F5" s="17"/>
-      <c r="G5" s="17"/>
+      <c r="E5" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="F5" s="18"/>
+      <c r="G5" s="18"/>
       <c r="H5" s="6"/>
       <c r="I5" s="6"/>
     </row>
@@ -1997,50 +2227,62 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="F6" s="4"/>
+        <v>27</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>28</v>
+      </c>
       <c r="G6" s="4"/>
-      <c r="H6" s="6"/>
-      <c r="I6" s="6"/>
+      <c r="H6" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="7" ht="67.5" spans="1:9">
       <c r="A7" s="4">
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D7" s="4"/>
       <c r="E7" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
-      <c r="H7" s="6"/>
-      <c r="I7" s="6"/>
+        <v>32</v>
+      </c>
+      <c r="F7" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="G7" s="19"/>
+      <c r="H7" s="20" t="s">
+        <v>34</v>
+      </c>
+      <c r="I7" s="9" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="8" spans="1:9">
       <c r="A8" s="4">
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="D8" s="4"/>
       <c r="E8" s="4"/>
@@ -2054,21 +2296,21 @@
         <v>8</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="C9" s="10" t="s">
         <v>10</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="F9" s="18" t="s">
-        <v>34</v>
-      </c>
-      <c r="G9" s="19"/>
+        <v>40</v>
+      </c>
+      <c r="F9" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="G9" s="21"/>
       <c r="H9" s="6"/>
       <c r="I9" s="6"/>
     </row>
@@ -2077,10 +2319,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="D10" s="4"/>
       <c r="E10" s="4"/>
@@ -2094,20 +2336,20 @@
         <v>10</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D11" s="15"/>
-      <c r="E11" s="20" t="s">
-        <v>38</v>
-      </c>
-      <c r="F11" s="15" t="s">
-        <v>39</v>
+      <c r="D11" s="14"/>
+      <c r="E11" s="22" t="s">
+        <v>45</v>
+      </c>
+      <c r="F11" s="23" t="s">
+        <v>46</v>
       </c>
       <c r="G11" s="4"/>
-      <c r="H11" s="21"/>
+      <c r="H11" s="24"/>
       <c r="I11" s="6"/>
     </row>
     <row r="12" ht="67.5" spans="1:9">
@@ -2115,20 +2357,20 @@
         <v>11</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D12" s="15"/>
-      <c r="E12" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="F12" s="15" t="s">
-        <v>42</v>
+      <c r="D12" s="14"/>
+      <c r="E12" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="F12" s="23" t="s">
+        <v>49</v>
       </c>
       <c r="G12" s="4"/>
-      <c r="H12" s="21"/>
+      <c r="H12" s="24"/>
       <c r="I12" s="6"/>
     </row>
     <row r="13" ht="40.5" spans="1:9">
@@ -2136,18 +2378,18 @@
         <v>12</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="F13" s="14"/>
+        <v>52</v>
+      </c>
+      <c r="F13" s="13"/>
       <c r="G13" s="4"/>
       <c r="H13" s="6"/>
       <c r="I13" s="6"/>
@@ -2157,136 +2399,154 @@
         <v>13</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D14" s="5"/>
       <c r="E14" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="H14" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="I14" s="6"/>
+        <v>54</v>
+      </c>
+      <c r="F14" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="G14" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="H14" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="I14" s="6" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="15" ht="67.5" spans="1:9">
       <c r="A15" s="4">
         <v>14</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="F15" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="G15" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="H15" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="I15" s="6"/>
+        <v>60</v>
+      </c>
+      <c r="F15" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="G15" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="H15" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="I15" s="6" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="16" ht="54" spans="1:9">
       <c r="A16" s="4">
         <v>15</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="F16" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="G16" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="H16" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="F16" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="G16" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="H16" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="I16" s="6"/>
+      <c r="I16" s="16" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="17" ht="67.5" spans="1:9">
       <c r="A17" s="4">
         <v>16</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D17" s="5"/>
       <c r="E17" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="F17" s="15"/>
-      <c r="G17" s="15"/>
-      <c r="H17" s="6"/>
-      <c r="I17" s="9"/>
+        <v>70</v>
+      </c>
+      <c r="F17" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="G17" s="14"/>
+      <c r="H17" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="I17" s="9" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="18" ht="40.5" spans="1:9">
       <c r="A18" s="4">
         <v>17</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D18" s="5"/>
       <c r="E18" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="F18" s="15"/>
-      <c r="G18" s="15"/>
-      <c r="H18" s="6"/>
-      <c r="I18" s="9"/>
+        <v>75</v>
+      </c>
+      <c r="F18" s="14" t="s">
+        <v>76</v>
+      </c>
+      <c r="G18" s="14"/>
+      <c r="H18" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="I18" s="9" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="19" ht="67.5" spans="1:9">
       <c r="A19" s="10">
         <v>18</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="C19" s="10" t="s">
         <v>10</v>
       </c>
       <c r="D19" s="10"/>
       <c r="E19" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="F19" s="22" t="s">
-        <v>68</v>
-      </c>
-      <c r="G19" s="23"/>
+        <v>79</v>
+      </c>
+      <c r="F19" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="G19" s="26"/>
       <c r="H19" s="6"/>
       <c r="I19" s="9"/>
     </row>
@@ -2295,19 +2555,19 @@
         <v>19</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>69</v>
+        <v>81</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="E20" s="14" t="s">
-        <v>71</v>
-      </c>
-      <c r="F20" s="24" t="s">
-        <v>72</v>
+        <v>82</v>
+      </c>
+      <c r="E20" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="F20" s="13" t="s">
+        <v>84</v>
       </c>
       <c r="G20" s="4"/>
       <c r="H20" s="6"/>
@@ -2318,19 +2578,19 @@
         <v>20</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>73</v>
+        <v>85</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="E21" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="F21" s="24" t="s">
-        <v>76</v>
+        <v>86</v>
+      </c>
+      <c r="E21" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="F21" s="13" t="s">
+        <v>88</v>
       </c>
       <c r="G21" s="4"/>
       <c r="H21" s="6"/>
@@ -2417,10 +2677,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="D3" s="4"/>
       <c r="E3" s="4"/>
@@ -2434,21 +2694,21 @@
         <v>3</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="C4" s="10" t="s">
         <v>10</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="F4" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="G4" s="13"/>
+        <v>40</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="G4" s="12"/>
       <c r="H4" s="6"/>
       <c r="I4" s="6"/>
     </row>
@@ -2457,10 +2717,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
@@ -2474,20 +2734,20 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D6" s="5"/>
       <c r="E6" s="8" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>48</v>
+        <v>89</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="H6" s="6"/>
       <c r="I6" s="6"/>
@@ -2497,22 +2757,22 @@
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="F7" s="14" t="s">
-        <v>54</v>
+        <v>60</v>
+      </c>
+      <c r="F7" s="13" t="s">
+        <v>90</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="H7" s="6"/>
       <c r="I7" s="6"/>
@@ -2522,22 +2782,22 @@
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="H8" s="6"/>
       <c r="I8" s="6"/>
@@ -2547,19 +2807,19 @@
         <v>8</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="C9" s="10" t="s">
         <v>10</v>
       </c>
       <c r="D9" s="10"/>
       <c r="E9" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="F9" s="14" t="s">
-        <v>77</v>
-      </c>
-      <c r="G9" s="15"/>
+        <v>79</v>
+      </c>
+      <c r="F9" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="G9" s="14"/>
       <c r="H9" s="6"/>
       <c r="I9" s="9"/>
     </row>
@@ -2578,5 +2838,6 @@
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: update hardware pin assignment workbook
</commit_message>
<xml_diff>
--- a/CIU32F003F5P6-TSSOP20.xlsx
+++ b/CIU32F003F5P6-TSSOP20.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="12375"/>
+    <workbookView windowWidth="28800" windowHeight="12375"/>
   </bookViews>
   <sheets>
     <sheet name="CIU32F003F5P6-TSSOP20" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="81">
   <si>
     <t>PIN</t>
   </si>
@@ -275,15 +275,6 @@
       <t>TIM1_CH2 
 TIM3_CH1</t>
     </r>
-  </si>
-  <si>
-    <t>Tim1_CH2</t>
-  </si>
-  <si>
-    <t>测试用，直接连在in2</t>
-  </si>
-  <si>
-    <t>PC1-&gt;PA7</t>
   </si>
   <si>
     <t>PB7</t>
@@ -333,15 +324,6 @@
       </rPr>
       <t>TIM1_CH4</t>
     </r>
-  </si>
-  <si>
-    <t>Tim1_ch4</t>
-  </si>
-  <si>
-    <t>测试用，跟随PWM_IN2,输出对应的占空比，频率16K</t>
-  </si>
-  <si>
-    <t>调试用，8P的脚刚好有电容</t>
   </si>
   <si>
     <t>VSS</t>
@@ -364,9 +346,6 @@
 MCO</t>
   </si>
   <si>
-    <t>SWDIO</t>
-  </si>
-  <si>
     <t>VDD</t>
   </si>
   <si>
@@ -711,13 +690,10 @@
     </r>
   </si>
   <si>
-    <t>TIm_ch1</t>
-  </si>
-  <si>
-    <t>测试用，直接连在in1</t>
-  </si>
-  <si>
-    <t>PA0--&gt;PB0</t>
+    <t>Tim1_ch1</t>
+  </si>
+  <si>
+    <t>输出同频率的pwm,用于调试</t>
   </si>
   <si>
     <t>PA1</t>
@@ -747,10 +723,7 @@
     </r>
   </si>
   <si>
-    <t>Tim1_ch3</t>
-  </si>
-  <si>
-    <t>测试用，跟随PWM_IN1,输出对应的占空比，频率16K</t>
+    <t>Tim1_ch2</t>
   </si>
   <si>
     <t>PA2</t>
@@ -763,7 +736,8 @@
 COMP2_OUT</t>
   </si>
   <si>
-    <t>SWCLK</t>
+    <t>SWCLK/
+UART1_RX</t>
   </si>
   <si>
     <t>PA3</t>
@@ -895,12 +869,6 @@
   <si>
     <t>UART1_RX
 /UART2_TX</t>
-  </si>
-  <si>
-    <t>TIM1_CH1</t>
-  </si>
-  <si>
-    <t>TIM1_CH2N</t>
   </si>
   <si>
     <t>SWCLK
@@ -1573,7 +1541,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1625,9 +1593,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2238,51 +2203,39 @@
       <c r="E6" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="F6" s="4" t="s">
-        <v>28</v>
-      </c>
+      <c r="F6" s="4"/>
       <c r="G6" s="4"/>
-      <c r="H6" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="I6" s="6" t="s">
-        <v>30</v>
-      </c>
+      <c r="H6" s="6"/>
+      <c r="I6" s="6"/>
     </row>
     <row r="7" ht="67.5" spans="1:9">
       <c r="A7" s="4">
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D7" s="4"/>
       <c r="E7" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="F7" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="G7" s="19"/>
-      <c r="H7" s="20" t="s">
-        <v>34</v>
-      </c>
-      <c r="I7" s="9" t="s">
-        <v>35</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="19"/>
+      <c r="I7" s="9"/>
     </row>
     <row r="8" spans="1:9">
       <c r="A8" s="4">
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="D8" s="4"/>
       <c r="E8" s="4"/>
@@ -2296,21 +2249,21 @@
         <v>8</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="C9" s="10" t="s">
         <v>10</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="F9" s="17" t="s">
-        <v>41</v>
-      </c>
-      <c r="G9" s="21"/>
+        <v>34</v>
+      </c>
+      <c r="F9" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="G9" s="20"/>
       <c r="H9" s="6"/>
       <c r="I9" s="6"/>
     </row>
@@ -2319,10 +2272,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="D10" s="4"/>
       <c r="E10" s="4"/>
@@ -2336,20 +2289,20 @@
         <v>10</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="14"/>
-      <c r="E11" s="22" t="s">
-        <v>45</v>
-      </c>
-      <c r="F11" s="23" t="s">
-        <v>46</v>
+      <c r="E11" s="21" t="s">
+        <v>38</v>
+      </c>
+      <c r="F11" s="22" t="s">
+        <v>39</v>
       </c>
       <c r="G11" s="4"/>
-      <c r="H11" s="24"/>
+      <c r="H11" s="23"/>
       <c r="I11" s="6"/>
     </row>
     <row r="12" ht="67.5" spans="1:9">
@@ -2357,20 +2310,20 @@
         <v>11</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D12" s="14"/>
       <c r="E12" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="F12" s="23" t="s">
-        <v>49</v>
+        <v>41</v>
+      </c>
+      <c r="F12" s="22" t="s">
+        <v>42</v>
       </c>
       <c r="G12" s="4"/>
-      <c r="H12" s="24"/>
+      <c r="H12" s="23"/>
       <c r="I12" s="6"/>
     </row>
     <row r="13" ht="40.5" spans="1:9">
@@ -2378,16 +2331,16 @@
         <v>12</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="F13" s="13"/>
       <c r="G13" s="4"/>
@@ -2399,23 +2352,23 @@
         <v>13</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D14" s="5"/>
       <c r="E14" s="8" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="G14" s="14" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="I14" s="6" t="s">
         <v>21</v>
@@ -2426,25 +2379,25 @@
         <v>14</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="G15" s="14" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="H15" s="9" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="I15" s="6" t="s">
         <v>21</v>
@@ -2455,22 +2408,22 @@
         <v>15</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="F16" s="15" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="G16" s="15" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="H16" s="16" t="s">
         <v>20</v>
@@ -2484,69 +2437,65 @@
         <v>16</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D17" s="5"/>
       <c r="E17" s="8" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="F17" s="14" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="G17" s="14"/>
       <c r="H17" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="I17" s="9" t="s">
-        <v>73</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="I17" s="9"/>
     </row>
     <row r="18" ht="40.5" spans="1:9">
       <c r="A18" s="4">
         <v>17</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D18" s="5"/>
       <c r="E18" s="8" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="F18" s="14" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="G18" s="14"/>
       <c r="H18" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="I18" s="9" t="s">
-        <v>35</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="I18" s="9"/>
     </row>
     <row r="19" ht="67.5" spans="1:9">
       <c r="A19" s="10">
         <v>18</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="C19" s="10" t="s">
         <v>10</v>
       </c>
       <c r="D19" s="10"/>
       <c r="E19" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="F19" s="25" t="s">
-        <v>80</v>
-      </c>
-      <c r="G19" s="26"/>
+        <v>70</v>
+      </c>
+      <c r="F19" s="24" t="s">
+        <v>71</v>
+      </c>
+      <c r="G19" s="25"/>
       <c r="H19" s="6"/>
       <c r="I19" s="9"/>
     </row>
@@ -2555,19 +2504,19 @@
         <v>19</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="E20" s="13" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="F20" s="13" t="s">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="G20" s="4"/>
       <c r="H20" s="6"/>
@@ -2578,19 +2527,19 @@
         <v>20</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="F21" s="13" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="G21" s="4"/>
       <c r="H21" s="6"/>
@@ -2677,10 +2626,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="D3" s="4"/>
       <c r="E3" s="4"/>
@@ -2694,18 +2643,18 @@
         <v>3</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="C4" s="10" t="s">
         <v>10</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="F4" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="F4" s="11" t="s">
         <v>24</v>
       </c>
       <c r="G4" s="12"/>
@@ -2717,10 +2666,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
@@ -2734,20 +2683,20 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D6" s="5"/>
       <c r="E6" s="8" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>89</v>
+        <v>48</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="H6" s="6"/>
       <c r="I6" s="6"/>
@@ -2757,22 +2706,22 @@
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="F7" s="13" t="s">
-        <v>90</v>
+        <v>54</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="H7" s="6"/>
       <c r="I7" s="6"/>
@@ -2782,22 +2731,22 @@
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="H8" s="6"/>
       <c r="I8" s="6"/>
@@ -2807,17 +2756,17 @@
         <v>8</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="C9" s="10" t="s">
         <v>10</v>
       </c>
       <c r="D9" s="10"/>
       <c r="E9" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="F9" s="13" t="s">
-        <v>91</v>
+        <v>70</v>
+      </c>
+      <c r="F9" s="11" t="s">
+        <v>80</v>
       </c>
       <c r="G9" s="14"/>
       <c r="H9" s="6"/>

</xml_diff>